<commit_message>
docs(remediation): apply S00-FINAL-HOTFIX for admin branch protection enforcement and DISC-004 numbering integrity
</commit_message>
<xml_diff>
--- a/التعلم/الاصلاح/Master_Remediation_Ledger_motion.xlsx
+++ b/التعلم/الاصلاح/Master_Remediation_Ledger_motion.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="103">
   <si>
     <t>CONFIRMED_ON_MAIN</t>
   </si>
@@ -319,6 +319,9 @@
   </si>
   <si>
     <t>[STATIC_CODE_EVIDENCE] scripts/pipeline.py and api/services implement duplicate gate orchestration logic</t>
+  </si>
+  <si>
+    <t>CHANGED — ENFORCE_ADMINS_PROTECTION_ENABLED_IN_S00: تم تفعيل حماية main بنجاح عبر GitHub API وتطبيقها على الجميع بما فيهم Admin/Owner (enforce_admins=true, PR required, 0 approving reviews, strict checks, no direct push, no force push).</t>
   </si>
 </sst>
 </file>
@@ -5663,7 +5666,7 @@
       </c>
       <c r="P83" s="8" t="str"/>
       <c r="Q83" s="8" t="s">
-        <v>89</v>
+        <v>102</v>
       </c>
       <c r="R83" s="8" t="str">
         <v>البند 82؛ يتطلب صلاحية إدارة</v>

</xml_diff>

<commit_message>
feat(security): enforce authentic HMAC-SHA256 bearer tokens and update package ownership roadmap (S02-SECURITY-CLOSURE)
- Implement Option B HMAC-SHA256 signed bearer token verification and issuance in api/core/auth.py
- Enforce strict signature verification prior to evaluating any payload claims
- Add 11 mandatory negative and tampering tests in tests/security/test_s02_negative_enforcement.py
- Reconcile future package ownership (STATE-001/LED-018 -> S03, CONC-001 -> S05, LED-005 -> S06, REC-001 -> S06, LED-008 -> S07, LED-054 -> S17) in reproductions, conftest, and Master Remediation Ledger
- Update ADR-002 and TRUST_MODEL.md with the canonical signed bearer token specification
</commit_message>
<xml_diff>
--- a/التعلم/الاصلاح/Master_Remediation_Ledger_motion.xlsx
+++ b/التعلم/الاصلاح/Master_Remediation_Ledger_motion.xlsx
@@ -1094,7 +1094,7 @@
       </c>
       <c r="N2" s="8" t="inlineStr">
         <is>
-          <t>يُعيّن عند البدء</t>
+          <t>S03</t>
         </is>
       </c>
       <c r="O2" s="8" t="inlineStr">
@@ -1280,7 +1280,7 @@
       </c>
       <c r="N4" s="8" t="inlineStr">
         <is>
-          <t>يُعيّن عند البدء</t>
+          <t>S05</t>
         </is>
       </c>
       <c r="O4" s="8" t="inlineStr">
@@ -1371,7 +1371,7 @@
       </c>
       <c r="N5" s="8" t="inlineStr">
         <is>
-          <t>يُعيّن عند البدء</t>
+          <t>S06</t>
         </is>
       </c>
       <c r="O5" s="8" t="inlineStr">
@@ -1462,7 +1462,7 @@
       </c>
       <c r="N6" s="8" t="inlineStr">
         <is>
-          <t>يُعيّن عند البدء</t>
+          <t>S06</t>
         </is>
       </c>
       <c r="O6" s="8" t="inlineStr">
@@ -1735,7 +1735,7 @@
       </c>
       <c r="N9" s="8" t="inlineStr">
         <is>
-          <t>يُعيّن عند البدء</t>
+          <t>S07</t>
         </is>
       </c>
       <c r="O9" s="8" t="inlineStr">
@@ -2613,7 +2613,7 @@
       </c>
       <c r="F19" s="8" t="inlineStr">
         <is>
-          <t>S09</t>
+          <t>S03</t>
         </is>
       </c>
       <c r="G19" s="8" t="inlineStr">
@@ -2653,7 +2653,7 @@
       </c>
       <c r="N19" s="8" t="inlineStr">
         <is>
-          <t>يُعيّن عند البدء</t>
+          <t>S03</t>
         </is>
       </c>
       <c r="O19" s="8" t="inlineStr">
@@ -5829,7 +5829,7 @@
       </c>
       <c r="N55" s="8" t="inlineStr">
         <is>
-          <t>يُعيّن عند البدء</t>
+          <t>S17</t>
         </is>
       </c>
       <c r="O55" s="8" t="inlineStr">

</xml_diff>

<commit_message>
feat(s16): pre-mount validation gate, canonical parseRenderInput & fail-closed contracts
</commit_message>
<xml_diff>
--- a/التعلم/الاصلاح/Master_Remediation_Ledger_motion.xlsx
+++ b/التعلم/الاصلاح/Master_Remediation_Ledger_motion.xlsx
@@ -4863,12 +4863,12 @@
       </c>
       <c r="M44" s="8" t="inlineStr">
         <is>
-          <t>لم يبدأ</t>
+          <t>مكتمل</t>
         </is>
       </c>
       <c r="N44" s="8" t="inlineStr">
         <is>
-          <t>يُعيّن عند البدء</t>
+          <t>S16</t>
         </is>
       </c>
       <c r="O44" s="8" t="inlineStr">
@@ -4950,12 +4950,12 @@
       </c>
       <c r="M45" s="8" t="inlineStr">
         <is>
-          <t>لم يبدأ</t>
+          <t>مكتمل</t>
         </is>
       </c>
       <c r="N45" s="8" t="inlineStr">
         <is>
-          <t>يُعيّن عند البدء</t>
+          <t>S16</t>
         </is>
       </c>
       <c r="O45" s="8" t="inlineStr">
@@ -5037,12 +5037,12 @@
       </c>
       <c r="M46" s="8" t="inlineStr">
         <is>
-          <t>لم يبدأ</t>
+          <t>مكتمل</t>
         </is>
       </c>
       <c r="N46" s="8" t="inlineStr">
         <is>
-          <t>يُعيّن عند البدء</t>
+          <t>S16</t>
         </is>
       </c>
       <c r="O46" s="8" t="inlineStr">
@@ -5124,12 +5124,12 @@
       </c>
       <c r="M47" s="8" t="inlineStr">
         <is>
-          <t>لم يبدأ</t>
+          <t>مكتمل</t>
         </is>
       </c>
       <c r="N47" s="8" t="inlineStr">
         <is>
-          <t>يُعيّن عند البدء</t>
+          <t>S16</t>
         </is>
       </c>
       <c r="O47" s="8" t="inlineStr">

</xml_diff>

<commit_message>
feat(s17): single authority build_render_input for local, docker, studio, and probe parity (LED-054)
</commit_message>
<xml_diff>
--- a/التعلم/الاصلاح/Master_Remediation_Ledger_motion.xlsx
+++ b/التعلم/الاصلاح/Master_Remediation_Ledger_motion.xlsx
@@ -5824,7 +5824,7 @@
       </c>
       <c r="M55" s="8" t="inlineStr">
         <is>
-          <t>لم يبدأ</t>
+          <t>مغلق</t>
         </is>
       </c>
       <c r="N55" s="8" t="inlineStr">
@@ -5837,8 +5837,16 @@
           <t>[AUTOMATED_RED_REPRODUCTION / RUNTIME_ENVIRONMENT_BLOCKED] pytest tests/remediation/reproductions/test_led_054_props_divergence.py --run-reproductions</t>
         </is>
       </c>
-      <c r="P55" s="8" t="str"/>
-      <c r="Q55" s="8" t="str"/>
+      <c r="P55" s="8" t="inlineStr">
+        <is>
+          <t>pytest tests/remediation/reproductions/test_led_054_props_divergence.py tests/core/test_s17_render_input.py tests/architecture/test_s17_architecture_guard.py tests/remediation/reproductions/test_s17_remediation_proof.py; vitest tests/remotion/s17_render_input_parity.test.ts</t>
+        </is>
+      </c>
+      <c r="Q55" s="8" t="inlineStr">
+        <is>
+          <t>CLOSED in S17: Canonical build_render_input authority in scripts/core/render_input.py used by Local, Docker, Studio, and Probe. Docker uses render_props.json identical to Local.</t>
+        </is>
+      </c>
       <c r="R55" s="8" t="inlineStr">
         <is>
           <t>B.7 ASSET-006; البند 54</t>

</xml_diff>

<commit_message>
feat(s18): canonical probe timing, review evidence bundle & mandatory contact sheet (LED-047..LED-050)
</commit_message>
<xml_diff>
--- a/التعلم/الاصلاح/Master_Remediation_Ledger_motion.xlsx
+++ b/التعلم/الاصلاح/Master_Remediation_Ledger_motion.xlsx
@@ -5211,12 +5211,12 @@
       </c>
       <c r="M48" s="8" t="inlineStr">
         <is>
-          <t>لم يبدأ</t>
+          <t>مكتمل</t>
         </is>
       </c>
       <c r="N48" s="8" t="inlineStr">
         <is>
-          <t>يُعيّن عند البدء</t>
+          <t>S18</t>
         </is>
       </c>
       <c r="O48" s="8" t="inlineStr">
@@ -5224,7 +5224,11 @@
           <t>[STATIC_CODE_EVIDENCE] scripts/gates/probe_qc.py:116 reads bp.get('timeline', []) which is empty in modern blueprints</t>
         </is>
       </c>
-      <c r="P48" s="8" t="str"/>
+      <c r="P48" s="8" t="inlineStr">
+        <is>
+          <t>tests/remediation/reproductions/test_s18_remediation_proof.py::test_proof_led_047_canonical_probe_timing</t>
+        </is>
+      </c>
       <c r="Q48" s="8" t="str"/>
       <c r="R48" s="8" t="inlineStr">
         <is>
@@ -5298,12 +5302,12 @@
       </c>
       <c r="M49" s="8" t="inlineStr">
         <is>
-          <t>لم يبدأ</t>
+          <t>مكتمل</t>
         </is>
       </c>
       <c r="N49" s="8" t="inlineStr">
         <is>
-          <t>يُعيّن عند البدء</t>
+          <t>S18</t>
         </is>
       </c>
       <c r="O49" s="8" t="inlineStr">
@@ -5311,7 +5315,11 @@
           <t>[STATIC_CODE_EVIDENCE] scripts/gates/probe_qc.py:111 reads bp.get('meta', {}).get('fps', 30) instead of root bp['fps']</t>
         </is>
       </c>
-      <c r="P49" s="8" t="str"/>
+      <c r="P49" s="8" t="inlineStr">
+        <is>
+          <t>tests/remediation/reproductions/test_s18_remediation_proof.py::test_proof_led_048_canonical_fps_authority</t>
+        </is>
+      </c>
       <c r="Q49" s="8" t="str"/>
       <c r="R49" s="8" t="inlineStr">
         <is>
@@ -5385,12 +5393,12 @@
       </c>
       <c r="M50" s="8" t="inlineStr">
         <is>
-          <t>لم يبدأ</t>
+          <t>مكتمل</t>
         </is>
       </c>
       <c r="N50" s="8" t="inlineStr">
         <is>
-          <t>يُعيّن عند البدء</t>
+          <t>S18</t>
         </is>
       </c>
       <c r="O50" s="8" t="inlineStr">
@@ -5398,7 +5406,11 @@
           <t>[STATIC_CODE_EVIDENCE] scripts/gates/probe_qc.py:202-210 catches contact sheet generation error and does not fail probe gate</t>
         </is>
       </c>
-      <c r="P50" s="8" t="str"/>
+      <c r="P50" s="8" t="inlineStr">
+        <is>
+          <t>tests/remediation/reproductions/test_s18_remediation_proof.py::test_proof_led_049_mandatory_contact_sheet_evidence</t>
+        </is>
+      </c>
       <c r="Q50" s="8" t="str"/>
       <c r="R50" s="8" t="inlineStr">
         <is>
@@ -5472,12 +5484,12 @@
       </c>
       <c r="M51" s="8" t="inlineStr">
         <is>
-          <t>لم يبدأ</t>
+          <t>مكتمل</t>
         </is>
       </c>
       <c r="N51" s="8" t="inlineStr">
         <is>
-          <t>يُعيّن عند البدء</t>
+          <t>S18</t>
         </is>
       </c>
       <c r="O51" s="8" t="inlineStr">
@@ -5485,7 +5497,11 @@
           <t>[STATIC_CODE_EVIDENCE] scripts/gates/probe_qc.py writes probe_qc_report.json but pipeline.py does not record hash in state</t>
         </is>
       </c>
-      <c r="P51" s="8" t="str"/>
+      <c r="P51" s="8" t="inlineStr">
+        <is>
+          <t>tests/remediation/reproductions/test_s18_remediation_proof.py::test_proof_led_050_review_bundle_evidence_chain</t>
+        </is>
+      </c>
       <c r="Q51" s="8" t="str"/>
       <c r="R51" s="8" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
fix(s19): enforce strict canonical final qc
</commit_message>
<xml_diff>
--- a/التعلم/الاصلاح/Master_Remediation_Ledger_motion.xlsx
+++ b/التعلم/الاصلاح/Master_Remediation_Ledger_motion.xlsx
@@ -5575,20 +5575,24 @@
       </c>
       <c r="M52" s="8" t="inlineStr">
         <is>
-          <t>لم يبدأ</t>
+          <t>مكتمل</t>
         </is>
       </c>
       <c r="N52" s="8" t="inlineStr">
         <is>
-          <t>يُعيّن عند البدء</t>
+          <t>S19</t>
         </is>
       </c>
       <c r="O52" s="8" t="inlineStr">
         <is>
-          <t>[STATIC_CODE_EVIDENCE] scripts/gates/final_qc.py:165-167 reads meta.get('aspect_ratio') and meta.get('duration_sec')</t>
-        </is>
-      </c>
-      <c r="P52" s="8" t="str"/>
+          <t>tests/remediation/reproductions/test_s19_reproductions.py::test_reproduce_led_051_duration_mismatch_and_fps_check</t>
+        </is>
+      </c>
+      <c r="P52" s="8" t="inlineStr">
+        <is>
+          <t>tests/remediation/reproductions/test_s19_remediation_proof.py::test_proof_led_051_canonical_aspect_ratios</t>
+        </is>
+      </c>
       <c r="Q52" s="8" t="str"/>
       <c r="R52" s="8" t="inlineStr">
         <is>
@@ -5662,20 +5666,24 @@
       </c>
       <c r="M53" s="8" t="inlineStr">
         <is>
-          <t>لم يبدأ</t>
+          <t>مكتمل</t>
         </is>
       </c>
       <c r="N53" s="8" t="inlineStr">
         <is>
-          <t>يُعيّن عند البدء</t>
+          <t>S19</t>
         </is>
       </c>
       <c r="O53" s="8" t="inlineStr">
         <is>
-          <t>[STATIC_CODE_EVIDENCE] scripts/gates/final_qc.py:73 check_av_sync is defined but never invoked in main()</t>
-        </is>
-      </c>
-      <c r="P53" s="8" t="str"/>
+          <t>tests/remediation/reproductions/test_s19_reproductions.py::test_reproduce_led_052_check_av_sync_is_called_in_execution_path</t>
+        </is>
+      </c>
+      <c r="P53" s="8" t="inlineStr">
+        <is>
+          <t>tests/remediation/reproductions/test_s19_remediation_proof.py::test_proof_led_052_av_sync_wired_into_real_execution_path</t>
+        </is>
+      </c>
       <c r="Q53" s="8" t="inlineStr">
         <is>
           <t>CONFIRMED_ON_MAIN (Rediscovered in S00 via DISC-006): check_av_sync is dead code never called in main()</t>
@@ -5753,20 +5761,24 @@
       </c>
       <c r="M54" s="8" t="inlineStr">
         <is>
-          <t>لم يبدأ</t>
+          <t>مكتمل</t>
         </is>
       </c>
       <c r="N54" s="8" t="inlineStr">
         <is>
-          <t>يُعيّن عند البدء</t>
+          <t>S19</t>
         </is>
       </c>
       <c r="O54" s="8" t="inlineStr">
         <is>
-          <t>[STATIC_CODE_EVIDENCE] scripts/gates/final_qc.py:70,142 catches exceptions and returns warning status</t>
-        </is>
-      </c>
-      <c r="P54" s="8" t="str"/>
+          <t>tests/remediation/reproductions/test_s19_reproductions.py::test_reproduce_led_053_analyzer_exceptions_use_check_failed_to_execute</t>
+        </is>
+      </c>
+      <c r="P54" s="8" t="inlineStr">
+        <is>
+          <t>tests/remediation/reproductions/test_s19_remediation_proof.py::test_proof_led_053_black_frame_analyzer_crash_is_check_failed_to_execute</t>
+        </is>
+      </c>
       <c r="Q54" s="8" t="str"/>
       <c r="R54" s="8" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
fix(s20): make remotion docker runtime hermetic
</commit_message>
<xml_diff>
--- a/التعلم/الاصلاح/Master_Remediation_Ledger_motion.xlsx
+++ b/التعلم/الاصلاح/Master_Remediation_Ledger_motion.xlsx
@@ -5947,21 +5947,29 @@
       </c>
       <c r="M56" s="8" t="inlineStr">
         <is>
-          <t>لم يبدأ</t>
+          <t>مكتمل</t>
         </is>
       </c>
       <c r="N56" s="8" t="inlineStr">
         <is>
-          <t>يُعيّن عند البدء</t>
+          <t>S20</t>
         </is>
       </c>
       <c r="O56" s="8" t="inlineStr">
         <is>
-          <t>[CONFIGURATION_EVIDENCE / RUNTIME_ENVIRONMENT_BLOCKED] .agents/docker/Dockerfile.remotion does not copy codebase; relies on host volume mount at runtime</t>
-        </is>
-      </c>
-      <c r="P56" s="8" t="str"/>
-      <c r="Q56" s="8" t="str"/>
+          <t>tests/remediation/reproductions/test_s20_reproductions.py::test_reproduce_led_055_dockerfile_hermetic_guarantees</t>
+        </is>
+      </c>
+      <c r="P56" s="8" t="inlineStr">
+        <is>
+          <t>pytest tests/architecture/test_s20_architecture_guard.py tests/remediation/reproductions/test_s20_reproductions.py tests/remediation/reproductions/test_s20_remediation_proof.py</t>
+        </is>
+      </c>
+      <c r="Q56" s="8" t="inlineStr">
+        <is>
+          <t>CLOSED in S20: Dockerfile.remotion is hermetic with node:20-bookworm base, locked npm ci, baked browser via remotion browser ensure, non-root user renderer (UID 1000), .dockerignore, and confined project data mounts. Verified local vs docker parity.</t>
+        </is>
+      </c>
       <c r="R56" s="8" t="inlineStr">
         <is>
           <t>البند 55</t>
@@ -5969,7 +5977,7 @@
       </c>
       <c r="S56" s="8" t="inlineStr">
         <is>
-          <t>4b96960</t>
+          <t>401dcc5</t>
         </is>
       </c>
     </row>

</xml_diff>